<commit_message>
feat(quotations): rebuild tariff and excel workbook using GIC actual operating routes and historical data
</commit_message>
<xml_diff>
--- a/BẢNG BÁO GIÁ DỊCH VỤ LOGISTICS - GIC.xlsx
+++ b/BẢNG BÁO GIÁ DỊCH VỤ LOGISTICS - GIC.xlsx
@@ -596,11 +596,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -640,7 +640,7 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>BÁO GIÁ CƯỚC VẬN CHUYỂN ĐƯỜNG BỘ</t>
+          <t>BÁO GIÁ CƯỚC VẬN CHUYỂN ĐƯỜNG BỘ - GIC LOGISTICS</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>1.9T
-4380*1850*1900m</t>
+4.38x1.85x1.9m</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -713,19 +713,19 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>高栏车 high-sided truck
+          <t>高栏车 high-sided
 Xe rào 14M</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>平坦车 flatbed truck
+          <t>平坦车 flatbed
 Xe sàn 14.3M</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>超地版 xe FOOC lùn
+          <t>超地版 xe FOOC
 Fooc lùn 18M</t>
         </is>
       </c>
@@ -739,49 +739,49 @@
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>春運貨場/Vietel物流园 Xuân Cương</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>北歌尔工厂 Goertek Bắc Ninh - KCN Quế Võ/Nam Sơn Hạp Linh</t>
+          <t>KCN Quế Võ / VSIP / Nam Sơn Hạp Linh (Bắc Ninh)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>2306000</v>
+        <v>2430000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2622200</v>
+        <v>2820000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>3035800</v>
+        <v>3200000</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3455900</v>
+        <v>3700000</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>4110900</v>
+        <v>4500000</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>4357600</v>
+        <v>4860000</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>4600000</v>
+        <v>4800000</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5830000</v>
+        <v>6080000</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>5830000</v>
+        <v>6400000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>7579000</v>
+        <v>8320000</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>7579000</v>
+        <v>8320000</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>12826000</v>
+        <v>13760000</v>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
@@ -792,49 +792,49 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>新清 Tân Thanh</t>
+          <t>Cửa khẩu Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>北歌尔工厂 Goertek Bắc Ninh - KCN Quế Võ/Nam Sơn Hạp Linh</t>
+          <t>Thuận Thành / Gia Bình (Bắc Ninh)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2407300</v>
+        <v>2470000</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>2739400</v>
+        <v>2860000</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>3174300</v>
+        <v>3250000</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>3605100</v>
+        <v>4982000</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4302500</v>
+        <v>4550000</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>4570500</v>
+        <v>4940000</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>5100000</v>
+        <v>4880000</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>6413000</v>
+        <v>6180000</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>6413000</v>
+        <v>6500000</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>8395200</v>
+        <v>8450000</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>8395200</v>
+        <v>8500000</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>13992000</v>
+        <v>14500000</v>
       </c>
       <c r="O7" s="10" t="inlineStr">
         <is>
@@ -845,102 +845,102 @@
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>芒街 Móng Cái</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>北歌尔工厂 Goertek Bắc Ninh - KCN Quế Võ/Nam Sơn Hạp Linh</t>
+          <t>Phú Thọ (KCN Thụy Vân / KCN Phú Thọ)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2847300</v>
+        <v>3120000</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>3248900</v>
+        <v>3610000</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>3776500</v>
+        <v>4100000</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>4253600</v>
+        <v>4760000</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>5136400</v>
+        <v>5740000</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>5496900</v>
+        <v>6230000</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>8500000</v>
+        <v>6150000</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11660000</v>
+        <v>7790000</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>11660000</v>
+        <v>8200000</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>15741000</v>
+        <v>10660000</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>15741000</v>
+        <v>10660000</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>26818000</v>
+        <v>17630000</v>
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>19h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>峙马 Chi Ma</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>北歌尔工厂 Goertek Bắc Ninh - KCN Quế Võ/Nam Sơn Hạp Linh</t>
+          <t>Vĩnh Phúc (KCN Khai Quang / Bình Xuyên)</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>2452700</v>
+        <v>2400000</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>2792000</v>
+        <v>2770000</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>3236600</v>
+        <v>3150000</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>3672200</v>
+        <v>3650000</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4388800</v>
+        <v>4410000</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>4666300</v>
+        <v>4790000</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>5300000</v>
+        <v>4720000</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>6646200</v>
+        <v>5980000</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>6646200</v>
+        <v>6300000</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>8745000</v>
+        <v>8190000</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>8745000</v>
+        <v>8190000</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>14575000</v>
+        <v>13540000</v>
       </c>
       <c r="O9" s="10" t="inlineStr">
         <is>
@@ -951,49 +951,49 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>锦寮 - 友谊关各货场 Pô Chai - Bãi xe hàng HNQL</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>北歌尔工厂 Goertek Bắc Ninh - KCN Quế Võ/Nam Sơn Hạp Linh</t>
+          <t>Hà Nội (KCN Thăng Long / Đài Tư / Gia Lâm / Long Biên)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2366800</v>
+        <v>2360000</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>2692500</v>
+        <v>2730000</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>3118800</v>
+        <v>3100000</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>3545400</v>
+        <v>3600000</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4225900</v>
+        <v>4340000</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>4485300</v>
+        <v>4800000</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5100000</v>
+        <v>4650000</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>6413000</v>
+        <v>5890000</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>6413000</v>
+        <v>6200000</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>8395200</v>
+        <v>8060000</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>8395200</v>
+        <v>8060000</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>13992000</v>
+        <v>13330000</v>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
@@ -1004,265 +1004,265 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>春運貨場/Vietel物流园 Xuân Cương</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>北歌尔分拨仓 Kho phân bố Goertek Nam Sơn Hạp Linh</t>
+          <t>Hải Dương (KCN Đại An / Nam Sách / Lai Vu)</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>2306000</v>
+        <v>2510000</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>2622200</v>
+        <v>2900000</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>3035800</v>
+        <v>3300000</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3455900</v>
+        <v>3830000</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4110900</v>
+        <v>4620000</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>4357600</v>
+        <v>5020000</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>4600000</v>
+        <v>4950000</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>5830000</v>
+        <v>6270000</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>5830000</v>
+        <v>6600000</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>7579000</v>
+        <v>8580000</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>7579000</v>
+        <v>8580000</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>12826000</v>
+        <v>14190000</v>
       </c>
       <c r="O11" s="10" t="inlineStr">
         <is>
-          <t>16h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>新清 Tân Thanh</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>北歌尔分拨仓 Kho phân bố Goertek Nam Sơn Hạp Linh</t>
+          <t>Hưng Yên (KCN Phố Nối A, B / Thăng Long 2)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>2407300</v>
+        <v>2470000</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2739400</v>
+        <v>2860000</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>3174300</v>
+        <v>3250000</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>3605100</v>
+        <v>3770000</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4302500</v>
+        <v>4600000</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>4570500</v>
+        <v>5000000</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5100000</v>
+        <v>4880000</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>6413000</v>
+        <v>6180000</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>6413000</v>
+        <v>6500000</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>8395200</v>
+        <v>8450000</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>8395200</v>
+        <v>8450000</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>13992000</v>
+        <v>13980000</v>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>16h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>芒街 Móng Cái</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>北歌尔分拨仓 Kho phân bố Goertek Nam Sơn Hạp Linh</t>
+          <t>Bắc Giang (KCN Đình Trám / Vân Trung / Quang Châu)</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>2847300</v>
+        <v>2090000</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>3248900</v>
+        <v>2420000</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>3776500</v>
+        <v>2750000</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>4253600</v>
+        <v>3190000</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5136400</v>
+        <v>3850000</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>5496900</v>
+        <v>4180000</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>8500000</v>
+        <v>4120000</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>11660000</v>
+        <v>5220000</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>11660000</v>
+        <v>5500000</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>15741000</v>
+        <v>7150000</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>15741000</v>
+        <v>7150000</v>
       </c>
       <c r="N13" s="9" t="n">
-        <v>26818000</v>
+        <v>11820000</v>
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>19h D+1</t>
+          <t>14h D+1</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>峙马 Chi Ma</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>北歌尔分拨仓 Kho phân bố Goertek Nam Sơn Hạp Linh</t>
+          <t>Thái Nguyên (KCN Yên Bình / Sông Công / Điềm Thụy)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2452700</v>
+        <v>2740000</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2792000</v>
+        <v>3170000</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>3236600</v>
+        <v>3600000</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3672200</v>
+        <v>4180000</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>4388800</v>
+        <v>5040000</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>4666300</v>
+        <v>5470000</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>5300000</v>
+        <v>5400000</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>6646200</v>
+        <v>6840000</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>6646200</v>
+        <v>7200000</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>8745000</v>
+        <v>9360000</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>8745000</v>
+        <v>9360000</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>14575000</v>
+        <v>15480000</v>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>16h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>锦寮 - 友谊关各货场 Pô Chai - Bãi xe hàng HNQL</t>
+          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>北歌尔分拨仓 Kho phân bố Goertek Nam Sơn Hạp Linh</t>
+          <t>Hải Phòng (KCN Đình Vũ / Tràng Duệ / Cảng Hải Phòng)</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>2366800</v>
+        <v>2850000</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>2692500</v>
+        <v>3300000</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>3118800</v>
+        <v>3750000</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>3545400</v>
+        <v>4350000</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>4225900</v>
+        <v>5250000</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>4485300</v>
+        <v>5700000</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>5100000</v>
+        <v>5620000</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>6413000</v>
+        <v>7120000</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>6413000</v>
+        <v>7500000</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>8395200</v>
+        <v>9750000</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>8395200</v>
+        <v>9750000</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>13992000</v>
+        <v>16120000</v>
       </c>
       <c r="O15" s="10" t="inlineStr">
         <is>
-          <t>16h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
@@ -1274,203 +1274,203 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>KCN Quế Võ / VSIP / Đại Đồng Hoàn Sơn (Bắc Ninh)</t>
+          <t>Thái Bình (KCN Phúc Khánh / TP. Thái Bình)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2350000</v>
+        <v>2850000</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>2650000</v>
+        <v>3300000</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>3100000</v>
+        <v>3750000</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>3500000</v>
+        <v>4350000</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>4200000</v>
+        <v>5250000</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>4450000</v>
+        <v>5700000</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>5000000</v>
+        <v>5620000</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>6400000</v>
+        <v>7120000</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>6400000</v>
+        <v>7500000</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>8300000</v>
+        <v>9800000</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>8300000</v>
+        <v>9750000</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>14000000</v>
+        <v>16120000</v>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>16h D+1</t>
+          <t>18h D+1</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>KCN Yên Bình / Sông Công (Thái Nguyên)</t>
+          <t>Thanh Hóa (KCN Bỉm Sơn / KCN Lễ Môn / Nghi Sơn)</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>2850000</v>
+        <v>4560000</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>3200000</v>
+        <v>5280000</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>3700000</v>
+        <v>6000000</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>4200000</v>
+        <v>6960000</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>5000000</v>
+        <v>9018000</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>5400000</v>
+        <v>9918000</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>6200000</v>
+        <v>9000000</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>7800000</v>
+        <v>11400000</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>7800000</v>
+        <v>12000000</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>9800000</v>
+        <v>15600000</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>9800000</v>
+        <v>15600000</v>
       </c>
       <c r="N17" s="9" t="n">
-        <v>16500000</v>
+        <v>25800000</v>
       </c>
       <c r="O17" s="10" t="inlineStr">
         <is>
-          <t>18h D+1</t>
+          <t>20h D+1</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
+          <t>Cửa khẩu Cốc Nam (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>KCN Đình Trám / Quang Châu / Vân Trung (Bắc Giang)</t>
+          <t>Hà Nội (Kho Gia Lâm / Phạm Ngọc Thạch / KCN Đài Tư)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>2100000</v>
+        <v>2360000</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>2400000</v>
+        <v>2730000</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>2800000</v>
+        <v>3100000</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>3200000</v>
+        <v>3600000</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>3800000</v>
+        <v>4400000</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>4100000</v>
+        <v>4710000</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>4600000</v>
+        <v>4650000</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>5800000</v>
+        <v>5890000</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>5800000</v>
+        <v>6200000</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>7500000</v>
+        <v>8060000</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>7500000</v>
+        <v>8060000</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>12500000</v>
+        <v>13330000</v>
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>14h D+1</t>
+          <t>16h D+1</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Cửa khẩu Hữu Nghị / Tân Thanh (Lạng Sơn)</t>
+          <t>Cửa khẩu Chi Ma (Lạng Sơn)</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Hà Nội (KCN Thăng Long / Đài Tư / Gia Lâm / Long Biên)</t>
+          <t>Hải Phòng (Cảng Đình Vũ) / Hà Nội</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>2500000</v>
+        <v>2740000</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2850000</v>
+        <v>3170000</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>3300000</v>
+        <v>3600000</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>3800000</v>
+        <v>4180000</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>4500000</v>
+        <v>5040000</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>4800000</v>
+        <v>5470000</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>5500000</v>
+        <v>5400000</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>7000000</v>
+        <v>6840000</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>7000000</v>
+        <v>7200000</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>9000000</v>
+        <v>9400000</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>9000000</v>
+        <v>9360000</v>
       </c>
       <c r="N19" s="9" t="n">
-        <v>15000000</v>
+        <v>15480000</v>
       </c>
       <c r="O19" s="10" t="inlineStr">
         <is>
@@ -1481,139 +1481,412 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Cửa khẩu Tân Thanh (Lạng Sơn)</t>
+          <t>Cảng Hải Phòng (Đình Vũ / Tân Vũ / Lạch Huyện)</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>KCN Thuận Thành / Gia Bình (Bắc Ninh)</t>
+          <t>Hà Nội / Hưng Yên / Vĩnh Phúc</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>2450000</v>
+        <v>1820000</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2750000</v>
+        <v>2110000</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>3200000</v>
+        <v>2400000</v>
       </c>
       <c r="F20" s="6" t="n">
+        <v>2780000</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>3360000</v>
+      </c>
+      <c r="H20" s="6" t="n">
         <v>3650000</v>
       </c>
-      <c r="G20" s="6" t="n">
-        <v>4350000</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>4600000</v>
-      </c>
       <c r="I20" s="6" t="n">
-        <v>5200000</v>
+        <v>3900000</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>6500000</v>
+        <v>4630000</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>6500000</v>
+        <v>4800000</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>8500000</v>
+        <v>6240000</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>8500000</v>
+        <v>6240000</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>14200000</v>
+        <v>10320000</v>
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>16h D+1</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+          <t>12h D+0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Đà Nẵng (KCN Hòa Khánh / Liên Chiểu)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>7030000</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>8140000</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>9250000</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>10730000</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>12950000</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>14060000</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>13880000</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>17580000</v>
+      </c>
+      <c r="K21" s="9" t="n">
+        <v>18500000</v>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>24050000</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <v>24050000</v>
+      </c>
+      <c r="N21" s="9" t="n">
+        <v>39780000</v>
+      </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>36h D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Nha Trang (Khánh Hòa)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>10560000</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>13920000</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>16800000</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>18240000</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>22800000</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>31200000</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>31200000</v>
+      </c>
+      <c r="N22" s="6" t="n">
+        <v>51600000</v>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>42h D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Đồng Nai (KCN Biên Hòa / Amata / Nhơn Trạch)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>13300000</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>15400000</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>17500000</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>20300000</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>24500000</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>26600000</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>26250000</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>33250000</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>45500000</v>
+      </c>
+      <c r="M23" s="9" t="n">
+        <v>45500000</v>
+      </c>
+      <c r="N23" s="9" t="n">
+        <v>75250000</v>
+      </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>48h D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>TP. Hồ Chí Minh (KCN Tân Bình / Cát Lái / Linh Trung)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>12540000</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>14520000</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>16500000</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>19140000</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>23100000</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>25080000</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>24750000</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>31350000</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>42900000</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>42900000</v>
+      </c>
+      <c r="N24" s="6" t="n">
+        <v>70950000</v>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>48h D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Cửa khẩu Tân Thanh / Hữu Nghị (Lạng Sơn)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Bà Rịa - Vũng Tàu (KCN Phú Mỹ / Cái Mép)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>13300000</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>15400000</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>17500000</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>20300000</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>24500000</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>26600000</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>26250000</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>33250000</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>45500000</v>
+      </c>
+      <c r="M25" s="9" t="n">
+        <v>45500000</v>
+      </c>
+      <c r="N25" s="9" t="n">
+        <v>75250000</v>
+      </c>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>48h D+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Ghi chú &amp; Điều khoản:</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>- Giá cước vận chuyển trên chưa bao gồm thuế giá trị gia tăng (VAT).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>- Phí lưu ca bắt đầu tính từ 15 giờ 00 phút ngày tiếp theo kể từ ngày đến nhận hàng/giao hàng:</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   + Phí lưu 02 ca đầu: 1.000.000 đ/ngày (xe tải) | 1.500.000 đ/ngày (xe container/fooc).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   + Phí lưu từ ca 3 đến ca 5: 1.500.000 đ/ngày (xe tải) | 2.000.000 đ/ngày (xe container/fooc).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   + Phí lưu ca thứ 6 trở đi: 2.000.000 đ/ngày.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>- Giá chưa bao gồm: phí bến bãi, bốc xếp, phí cân xe, nâng hạ hàng hóa, phí thủ tục xuất nhập cảnh.</t>
+          <t>- Giá cước vận chuyển trên chưa bao gồm thuế giá trị gia tăng (VAT 8% hoặc 10%).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>- Giá đã bao gồm phí cầu đường bộ, lương lái xe, chi phí nhiên liệu (dầu diesel).</t>
+          <t>- Bảng giá được xây dựng trên cơ sở dữ liệu vận hành thực tế các tuyến vận chuyển chính thức của GIC Logistics.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>- Trường hợp hủy chuyến: Nếu xe đã điều đến bãi đóng hàng hoặc đi được nửa đường, khách hàng thanh toán 50% cước phí.</t>
+          <t>- Phí lưu ca bắt đầu tính từ 15 giờ 00 phút ngày tiếp theo kể từ ngày đến nhận hàng/giao hàng:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>- Khi giá dầu diesel có sự biến động +/- 10%, giá cước sẽ được hai bên điều chỉnh hiệp thương lại.</t>
+          <t xml:space="preserve">   + Phí lưu 02 ca đầu: 1.000.000 đ/ngày (xe tải thùng) | 1.500.000 đ/ngày (xe container/fooc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   + Phí lưu từ ca 3 đến ca 5: 1.500.000 đ/ngày (xe tải thùng) | 2.000.000 đ/ngày (xe container/fooc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   + Phí lưu ca thứ 6 trở đi: 2.000.000 đ/ngày.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>- Giá đã bao gồm: phí cầu đường bộ, lương lái xe, chi phí nhiên liệu (dầu diesel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>- Giá chưa bao gồm: phí bến bãi, bốc xếp, phí cân xe, nâng hạ hàng hóa, lệ phí thủ tục xuất nhập cảnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>- Trường hợp hủy chuyến: Nếu xe đã điều đến nhà máy hoặc lăn bánh được nửa đường, khách hàng thanh toán 50% cước phí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>- Khi giá dầu diesel thị trường có sự biến động +/- 10%, giá cước sẽ được hai bên hiệp thương điều chỉnh lại.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="B26:O26"/>
+  <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B27:O27"/>
-    <mergeCell ref="B24:O24"/>
+    <mergeCell ref="B35:O35"/>
     <mergeCell ref="B30:O30"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="B29:O29"/>
-    <mergeCell ref="B25:O25"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="B22:O22"/>
+    <mergeCell ref="B33:O33"/>
+    <mergeCell ref="B31:O31"/>
+    <mergeCell ref="B36:O36"/>
+    <mergeCell ref="B34:O34"/>
     <mergeCell ref="B28:O28"/>
-    <mergeCell ref="B23:O23"/>
     <mergeCell ref="A4:O4"/>
+    <mergeCell ref="B32:O32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1692,7 +1965,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Cơ Sở &amp; Ghi Chú Kỹ Thuật</t>
+          <t>Cơ Sở Dữ Liệu Thực Tế</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1993,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Định mức nhân công dỡ hàng nặng tại kho bãi Lạng Sơn và Hub giao hàng.</t>
+          <t>Căn cứ chi phí nhân công bốc dỡ thực tế tại kho Đồng Đăng, Lạng Sơn và các Hub.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +2021,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Áp dụng cho lô hàng từ 3 tấn trở lên, sang xe hoặc dỡ vào kho.</t>
+          <t>Áp dụng cho lô hàng từ 3 tấn trở lên, sang xe hoặc dỡ vào kho khách.</t>
         </is>
       </c>
     </row>
@@ -1776,7 +2049,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Hàng nhẹ thể tích (carton, bao bì, bông sợi). Bốc xếp bán kính ≤ 15m.</t>
+          <t>Hàng nhẹ thể tích (carton, bao bì, gia dụng). Bốc xếp bán kính tiêu chuẩn ≤ 15m.</t>
         </is>
       </c>
     </row>
@@ -1804,7 +2077,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ thực tế bốc dỡ hàng xe 5T tại kho Lạng Sơn (Lô CP 5.0).</t>
+          <t>Căn cứ thực tế sang hàng xe 5T hàng Keep Rise ở Lạng Sơn (Giá vốn 900.000 đ).</t>
         </is>
       </c>
     </row>
@@ -1832,7 +2105,7 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Định mức nhân công bốc dỡ nguyên xe tải 8 tấn (thời gian dưới 3 giờ).</t>
+          <t>Căn cứ thực tế bốc xếp hạ kho hoặc sang xe trọn gói cho xe 8T tại Đồng Đăng.</t>
         </is>
       </c>
     </row>
@@ -1888,7 +2161,7 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ dữ liệu thực tế bốc dỡ hàng nguyên container (Lô 2 tháng 09/2026).</t>
+          <t>Căn cứ 8 đợt dỡ hàng nguyên container thực tế (Giá vốn TB 3.992.500 đ, Bán 4.651.286 đ).</t>
         </is>
       </c>
     </row>
@@ -1916,7 +2189,7 @@
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ 5 đợt sang hàng pallet thực tế (Lô CP 2.0). Bao gồm kéo và cố định.</t>
+          <t>Căn cứ 5 đợt cơ giới sang hàng pallet thực tế (Lô CP 2.0). Bao gồm kéo và cố định.</t>
         </is>
       </c>
     </row>
@@ -1944,7 +2217,7 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Thuê xe nâng cơ giới sang tải kiện hàng nặng trên 500kg tại bãi cửa khẩu.</t>
+          <t>Căn cứ thực tế thuê xe nâng cơ giới sang tải tại bãi Lạng Sơn (Giá vốn 859.090 đ).</t>
         </is>
       </c>
     </row>
@@ -1972,7 +2245,7 @@
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Vé bến bãi vào khu vực sang tải Lạng Sơn (Lô CP 5.0).</t>
+          <t>Vé bến bãi vào khu vực sang tải Lạng Sơn thực tế (90.000 đ - 240.000 đ, TB 140.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2273,7 @@
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>Thực tế bốc xếp giao hàng chuỗi Keep tại Hà Nội gồm xe nội thành và dỡ hàng.</t>
+          <t>Căn cứ chi phí thực tế bốc xếp giao hàng chuỗi Keep tại Hà Nội (Giá vốn 1.000.000 đ - 3.240.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2301,7 @@
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>Chi phí bốc xếp giao hàng thực tế tại kho và cửa hàng TP.HCM.</t>
+          <t>Căn cứ chi phí thực tế bốc xếp giao hàng tại HCM (Giá vốn 2.000.000 đ/chuyến).</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2329,7 @@
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
-          <t>Chi phí thực tế bốc xếp lên cửa hàng và giao hàng tại Nha Trang.</t>
+          <t>Căn cứ chi phí thực tế bốc xếp lên cửa hàng và giao hàng Keep ở Nha Trang (Giá vốn 1.000.000 đ - 2.300.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2357,7 @@
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>Chi phí thực tế bốc xếp giao hàng tại Vũng Tàu.</t>
+          <t>Căn cứ chi phí thực tế bốc xếp giao hàng Keep Rise ở Vũng Tàu (Giá vốn 400.000 đ - 1.500.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2385,7 @@
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
-          <t>Chi phí thực tế bốc xếp giao hàng tại Đà Nẵng.</t>
+          <t>Căn cứ chi phí thực tế bốc xếp giao hàng Keep Rise ở Đà Nẵng (Giá vốn 800.000 đ/chuyến).</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2413,7 @@
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Chi phí thuê kho và bốc xếp hàng phân phối tại Đà Lạt.</t>
+          <t>Căn cứ chi phí thực tế thuê kho và bốc xếp hàng Keep Rise tại Đà Lạt (Giá vốn 8.300.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2152,14 +2425,14 @@
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>- Giá chưa bao gồm VAT (8% hoặc 10%). Phạm vi di chuyển bốc xếp thủ công tiêu chuẩn ≤ 15m tính từ mép sàn xe.</t>
+          <t>- Giá chưa bao gồm VAT. Phạm vi di chuyển bốc xếp thủ công tiêu chuẩn ≤ 15m tính từ mép sàn xe.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>- Trường hợp hàng quá khổ, kiện máy trên 1 tấn yêu cầu sử dụng xe cẩu tự hành hoặc xe nâng chuyên dụng sẽ báo giá cụ thể theo vị trí hiện trường.</t>
+          <t>- Trường hợp hàng quá khổ, kiện máy trên 1 tấn yêu cầu xe cẩu tự hành sẽ báo giá riêng theo vị trí hiện trường.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2441,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B24:F24"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
@@ -2182,7 +2455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2249,7 +2522,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Cơ Sở Dữ Liệu &amp; Quy Định</t>
+          <t>Cơ Sở Dữ Liệu Thực Tế</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2550,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ các tờ khai A11 thực tế (Sunluxe). Bao gồm lập tờ khai nháp, truyền VNACCS, kiểm tra C/O, làm thủ tục hiện trường.</t>
+          <t>Căn cứ các tờ khai A11 thực tế thông quan (Sunluxe, Ween, Hưng Đại). Bao gồm lên tờ khai nháp, truyền VNACCS, kiểm tra chứng từ, thông quan.</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2578,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ các tờ khai A12 thực tế (Sunluxe). Áp dụng doanh nghiệp nhập nguyên phụ liệu sản xuất.</t>
+          <t>Căn cứ các tờ khai A12 thực tế thông quan (Sunluxe). Áp dụng doanh nghiệp nhập nguyên phụ liệu sản xuất.</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2593,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Loại hình E21 (Gia công cho thương nhân nước ngoài)</t>
+          <t>Loại hình E21 (Gia công thương nhân nước ngoài)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -2333,7 +2606,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ tờ khai E21 thực tế thông quan. Áp dụng hợp đồng gia công miễn thuế NK.</t>
+          <t>Căn cứ tờ khai E21 thực tế đã thông quan. Áp dụng hợp đồng gia công miễn thuế nhập khẩu.</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2634,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ tờ khai H11 thực tế. Áp dụng cho hàng phi mậu dịch, hàng mẫu không thanh toán.</t>
+          <t>Căn cứ tờ khai H11 thực tế đã thông quan. Áp dụng cho hàng phi mậu dịch, hàng mẫu không thanh toán.</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2662,7 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ tờ khai G13 thực tế. Áp dụng hàng tạm nhập phục vụ sự kiện, triển lãm.</t>
+          <t>Căn cứ tờ khai G13 thực tế đã thông quan. Áp dụng hàng tạm nhập phục vụ sự kiện, triển lãm.</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2690,7 @@
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ tờ khai A41 thực tế. Doanh nghiệp chế xuất bán vào nội địa hoặc mua hàng nội địa.</t>
+          <t>Căn cứ tờ khai A41 thực tế đã thông quan. Doanh nghiệp chế xuất bán vào nội địa hoặc mua hàng nội địa.</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2700,12 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Dịch vụ Tờ khai Hải quan - Lô hàng lẻ / Cont 20 tiêu chuẩn</t>
+          <t>Phí tờ khai hải quan và hiện trường (Kaixin, Sao Đỏ)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Tờ khai thông thường (Lô lẻ / 1 Cont 20 ≤ 3 dòng)</t>
+          <t>Làm thủ tục hải quan &amp; trực tiếp tại hiện trường</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -2441,11 +2714,11 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>2500000</v>
+        <v>3250000</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ &gt;30 đợt DVTK HQ thực tế trong hệ thống (Lô 1 tháng 08/2026).</t>
+          <t>Căn cứ phí làm thủ tục hải quan và hiện trường thực tế đã thu khách Kaixin, Sao Đỏ.</t>
         </is>
       </c>
     </row>
@@ -2455,25 +2728,25 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Phụ thu Tờ khai nhánh (Từ dòng hàng thứ 5 trở đi)</t>
+          <t>Dịch vụ Tờ khai Hải quan - Lô hàng lẻ / Cont 20 tiêu chuẩn</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Tờ khai nhánh (&gt;4 dòng hàng theo quy định VNACCS)</t>
+          <t>Tờ khai thông thường (Lô lẻ / 1 Cont 20 ≤ 3 dòng)</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Tờ khai nhánh</t>
+          <t>Tờ khai</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>200000</v>
+        <v>2500000</v>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Định mức phụ thu tờ khai nhánh trên hệ thống VNACCS khi lô hàng có trên 4 dòng.</t>
+          <t>Căn cứ &gt;30 đợt làm DVTK HQ thực tế trong hệ thống GIC (Giá vốn TB 1.980.000 đ, Giá bán 2.500.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2483,25 +2756,25 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Phí tiếp nhận hồ sơ &amp; Xử lý tờ khai quay đầu</t>
+          <t>Tách hồ sơ + Hải quan giám sát cơ động</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Hồ sơ quay đầu chuyển cửa khẩu</t>
+          <t>Tách hồ sơ và giám sát hải quan cơ động</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Bộ hồ sơ</t>
+          <t>Lô/Đợt</t>
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ cước thực tế tiếp nhận hồ sơ quay đầu và làm thủ tục chuyển cửa khẩu (Cột 26 Báo Cáo Bán Hàng).</t>
+          <t>Căn cứ chi phí tách hồ sơ và giám sát cơ động thực tế phát sinh tại bến bãi cửa khẩu.</t>
         </is>
       </c>
     </row>
@@ -2511,55 +2784,103 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
+          <t>Phụ thu Tờ khai nhánh (Từ dòng hàng thứ 5 trở đi)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Tờ khai nhánh (&gt;4 dòng hàng theo quy định VNACCS)</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Tờ khai nhánh</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Định mức phụ thu tờ khai nhánh theo quy định hệ thống VNACCS/VCIS khi lô hàng có trên 4 dòng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Phí tiếp nhận hồ sơ &amp; Xử lý tờ khai quay đầu</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Hồ sơ quay đầu chuyển cửa khẩu</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Bộ hồ sơ</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Căn cứ cước thực tế tiếp nhận hồ sơ quay đầu và làm thủ tục chuyển cửa khẩu (Cột 26 Báo Cáo Bán Hàng).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
           <t>Phí Hải quan giám sát tại bến bãi cửa khẩu</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Hải quan giám sát bãi kiểm hóa</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Xe/Cont</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E17" s="18" t="n">
         <v>400000</v>
       </c>
-      <c r="F15" s="19" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>Căn cứ chi phí hải quan giám sát thực tế tại bãi kiểm hóa Tân Thanh/Hữu Nghị.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Ghi chú:</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>- Đơn giá dịch vụ hải quan chưa bao gồm các khoản thuế nhập khẩu, thuế GTGT hàng nhập khẩu và lệ phí nhà nước.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>- Đã bao gồm chi phí kiểm tra bộ chứng từ (Invoice, Packing List, C/O), lên tờ khai nháp và thông quan luồng Xanh/Vàng.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B19:F19"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2571,7 +2892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2638,7 +2959,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Cơ Sở Dữ Liệu &amp; Quy Định</t>
+          <t>Cơ Sở Dữ Liệu Thực Tế</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2987,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ kiểm tra chất lượng thực tế thiết bị gia dụng tại Quatest 1 (Lô 08.2026).</t>
+          <t>Căn cứ 3 đợt kiểm tra chất lượng thực tế tại Quatest 1 (Lô 08.2026: Giá vốn 3.250.000 đ, Giá thu 4.000.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2722,7 +3043,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ chi phí Quatest thực tế hàng Keep Rise (thử nghiệm Formaldehyd &amp; Azo).</t>
+          <t>Căn cứ chi phí Quatest thực tế hàng Keep Rise (thử nghiệm Formaldehyd &amp; Amin thơm Azo, Giá vốn 5.000.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2750,7 +3071,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Định mức thử nghiệm chứng nhận hợp quy đồ chơi và đồ dùng tiếp xúc thực phẩm.</t>
+          <t>Định mức thử nghiệm chứng nhận hợp quy đồ chơi trẻ em và đồ dùng tiếp xúc thực phẩm.</t>
         </is>
       </c>
     </row>
@@ -2778,7 +3099,7 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Chi phí lấy mẫu sớm tại bãi kiểm hóa Lạng Sơn gửi về phòng lab (Lô CP 5.0).</t>
+          <t>Căn cứ chi phí lấy mẫu sớm tại bãi kiểm hóa Lạng Sơn (Giá vốn 1.000.000 đ - 1.500.000 đ, Lô CP 5.0).</t>
         </is>
       </c>
     </row>
@@ -2806,7 +3127,7 @@
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>Phí soạn hồ sơ, dịch thuật chứng chỉ và nộp NSW (Lô 08.2026).</t>
+          <t>Phí soạn đơn đăng ký, dịch thuật chứng chỉ và nộp cổng thông tin NSW (Lô 08.2026).</t>
         </is>
       </c>
     </row>
@@ -2834,7 +3155,7 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ 22 lượt kiểm dịch y tế thực tế tại cửa khẩu Hữu Nghị/Tân Thanh.</t>
+          <t>Căn cứ 22 lượt kiểm dịch y tế thực tế tại cửa khẩu Hữu Nghị/Tân Thanh (Giá vốn 25.000 đ - 165.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2862,7 +3183,7 @@
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ 8 lượt kiểm dịch y tế xe phía Trung Quốc thực tế.</t>
+          <t>Căn cứ 8 lượt kiểm dịch y tế xe phía Trung Quốc thực tế (Giá vốn 25.000 đ - 75.000 đ).</t>
         </is>
       </c>
     </row>
@@ -2872,7 +3193,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Hải quan &amp; Giám định đồng bộ dây chuyền máy móc</t>
+          <t>Chi phí Hải quan &amp; Giám định đồng bộ dây chuyền máy móc</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2890,7 +3211,7 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ chi phí hải quan và giám định đồng bộ Vinacontrol/FCC (Lô 08.2026).</t>
+          <t>Căn cứ chi phí hải quan và giám định đồng bộ Vinacontrol/FCC thực tế thu khách (8.000.000 đ/lô, Lô 08.2026).</t>
         </is>
       </c>
     </row>
@@ -2918,7 +3239,7 @@
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Phí soạn thảo bộ hồ sơ kỹ thuật giám định đồng bộ dây chuyền.</t>
+          <t>Phí chuẩn bị hồ sơ kỹ thuật giám định đồng bộ thực tế đã thu khách (500.000 đ/bộ, Lô 08.2026).</t>
         </is>
       </c>
     </row>
@@ -2946,29 +3267,16 @@
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>Thực tế xử lý kiểm định đồng bộ tại cảng/cửa khẩu (Lô 08.2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Ghi chú:</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>- Phí kiểm tra chất lượng áp dụng cho mẫu thông thường. Mẫu yêu cầu phá hủy hoặc thử nghiệm chuyên sâu sẽ theo biểu phí cơ quan kiểm định.</t>
+          <t>Thực tế xử lý kiểm định đồng bộ tại cảng/cửa khẩu đã thu khách (3.000.000 đ - 3.500.000 đ/lô).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3047,7 +3355,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Cơ Sở Quy Định &amp; Ghi Chú</t>
+          <t>Cơ Sở Dữ Liệu Thực Tế</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3383,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Căn cứ biên lai nộp phí sử dụng hạ tầng cửa khẩu Lạng Sơn (Lô 1, Lô 2).</t>
+          <t>Căn cứ biên lai nộp phí sử dụng hạ tầng cửa khẩu Lạng Sơn thực tế (Giá vốn 859.273 đ, Giá thu 1.389.000 đ).</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3411,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Căn cứ biểu mức thu phí hạ tầng cửa khẩu áp dụng phương tiện container nhập khẩu.</t>
+          <t>Căn cứ biểu mức thu phí hạ tầng cửa khẩu Hữu Nghị / Tân Thanh áp dụng container nhập khẩu.</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3439,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Vé xe bến bãi thực tế cổng kiểm soát Tân Thanh và Hữu Nghị.</t>
+          <t>Vé xe bến bãi thực tế ra vào cổng kiểm soát Tân Thanh và Hữu Nghị (Giá vốn 147.273 đ - 250.000 đ).</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3467,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Chi phí thực tế đóng dấu đầu xe và cấp tem kiểm soát phương tiện qua biên giới.</t>
+          <t>Chi phí thực tế đóng dấu đầu xe và cấp tem kiểm soát phương tiện qua biên giới (Giá vốn 100.000 đ - 150.000 đ).</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3495,7 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Dữ liệu thực tế phí lưu ca xe tải trong các lô hàng GIC (1.000.000 đ/ngày đêm).</t>
+          <t>Dữ liệu thực tế phí lưu ca xe tải trong các lô hàng GIC (1.000.000 đ/ngày đêm, Cột 18 Báo Cáo Bán Hàng).</t>
         </is>
       </c>
     </row>
@@ -3225,12 +3533,12 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Phụ phí phát sinh thêm điểm trả hàng (Nội tỉnh)</t>
+          <t>Phụ phí phát sinh thêm 1 điểm giao hàng (Thái Bình / Hải Phòng)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Điểm trả hàng thứ 2 trong cùng tỉnh/thành (≤20km)</t>
+          <t>Điểm trả hàng ngoại tỉnh (Cách tuyến chính &gt;30km)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -3239,11 +3547,11 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Chi phí phát sinh điều động xe trả thêm hàng tại điểm thứ 2 nội tỉnh.</t>
+          <t>Căn cứ 3 đợt phát sinh thực tế giao thêm 1 điểm tại Thái Bình và Hải Phòng đã thu khách (1.000.000 đ/điểm).</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3561,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Phụ phí phát sinh thêm điểm trả hàng (Ngoại tỉnh lân cận)</t>
+          <t>Phụ phí phát sinh thêm điểm trả hàng (Nội tỉnh)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Điểm trả hàng ngoại tỉnh (Cách tuyến &gt;30km)</t>
+          <t>Điểm trả hàng thứ 2 trong cùng tỉnh/thành (≤20km)</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -3267,11 +3575,11 @@
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Thực tế phát sinh giao thêm 1 điểm tại Thái Bình/Hải Phòng (Lô 08.2026).</t>
+          <t>Chi phí phát sinh điều động xe trả thêm hàng tại điểm thứ 2 nội tỉnh.</t>
         </is>
       </c>
     </row>
@@ -3299,7 +3607,7 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Khoản phí bồi hoàn hủy xe đột xuất khi phương tiện đã tập kết bến bãi.</t>
+          <t>Căn cứ thực tế khoản phí hủy xe Tân Thanh - Thuận Thành đã thu khách (1.000.000 đ/chuyến).</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3675,7 @@
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>